<commit_message>
Refresh comp_table.xlsx with current market data
Prices moved higher across the board since prior run; KNSL up to $370.30
from $310.66. Ranking of KNSL vs peers unchanged.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comp_table.xlsx
+++ b/comp_table.xlsx
@@ -603,7 +603,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>yfinance data pulled 2026-06-12 00:23:01.  EDGAR ROE columns are TTM through 2026-03-31 (latest 10-Q).</t>
+          <t>yfinance data pulled 2026-07-28 23:01:12.  EDGAR ROE columns are TTM through 2026-03-31, 2026-06-30 (latest 10-Q).</t>
         </is>
       </c>
     </row>
@@ -686,37 +686,37 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>7.164695552</v>
+        <v>8.433939455999999</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>310.66</v>
+        <v>370.26</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>13.679437</v>
+        <v>14.663763</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>14.301748</v>
+        <v>17.10468</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>3.641807568165437</v>
+        <v>4.144209835910912</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>3.641807568165437</v>
+        <v>4.144209835910912</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>0.102</v>
+        <v>0.168</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.2896014088844931</v>
+        <v>0.2855374539010263</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>0.2815630067499332</v>
+        <v>0.27788107091471</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>0.27484</v>
+        <v>0.28492</v>
       </c>
       <c r="M5" s="10" t="n">
-        <v>0.32</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="6">
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>3.051920896</v>
+        <v>3.794294528</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>115.15</v>
+        <v>143.16</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>16.059973</v>
+        <v>19.664835</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>10.298389</v>
+        <v>12.85251</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>3.182269851382478</v>
+        <v>3.956350605137017</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>3.182269851382478</v>
+        <v>3.956350605137017</v>
       </c>
       <c r="I6" s="15" t="n">
         <v>0.597</v>
@@ -776,37 +776,37 @@
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>4.976621568</v>
+        <v>5.974422016</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>54.13</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>12.617716</v>
+        <v>13.450413</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>19.491276</v>
+        <v>24.085596</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>2.770345842495227</v>
+        <v>3.409834409271081</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>2.843250846698447</v>
+        <v>3.501897078226761</v>
       </c>
       <c r="I7" s="15" t="n">
-        <v>0.04</v>
+        <v>0.152</v>
       </c>
       <c r="J7" s="15" t="n">
-        <v>0.2247521659695697</v>
+        <v>0.2501410659324598</v>
       </c>
       <c r="K7" s="15" t="n">
-        <v>0.2111178952517287</v>
+        <v>0.2358963204249953</v>
       </c>
       <c r="L7" s="15" t="n">
-        <v>0.20805</v>
+        <v>0.22219</v>
       </c>
       <c r="M7" s="16" t="n">
-        <v>1.33</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="8">
@@ -821,25 +821,25 @@
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>25.143570432</v>
+        <v>28.26348544</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>67.54000000000001</v>
+        <v>76.17</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>14.309323</v>
+        <v>15.672839</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>13.998798</v>
+        <v>15.769044</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>2.581594676550765</v>
+        <v>2.901929292421108</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>2.63139683804179</v>
+        <v>2.957911105743479</v>
       </c>
       <c r="I8" s="15" t="n">
-        <v>0.04</v>
+        <v>0.012</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>0.1977587555310215</v>
@@ -848,10 +848,10 @@
         <v>0.1863939752904686</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>0.12639</v>
+        <v>0.12943</v>
       </c>
       <c r="M8" s="16" t="n">
-        <v>0.59</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="9">
@@ -866,22 +866,22 @@
         </is>
       </c>
       <c r="C9" s="12" t="n">
-        <v>22.900088832</v>
+        <v>25.519835136</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>1830</v>
+        <v>2039.35</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>13.244554</v>
+        <v>14.577198</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>15.032036</v>
+        <v>17.436798</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>1.262966664758436</v>
+        <v>1.407448735389214</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>1.659792843580859</v>
+        <v>1.849671415636899</v>
       </c>
       <c r="I9" s="15" t="n">
         <v>-0.169</v>
@@ -911,22 +911,22 @@
         </is>
       </c>
       <c r="C10" s="12" t="n">
-        <v>7.338410496</v>
+        <v>8.792969215999999</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>99.54000000000001</v>
+        <v>119.27</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>7.4394617</v>
+        <v>8.75055</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>6.858277</v>
+        <v>8.234097500000001</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>1.150106430769597</v>
+        <v>1.378070965966402</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>1.193143579594712</v>
+        <v>1.429638580638532</v>
       </c>
       <c r="I10" s="15" t="n">
         <v>0.08</v>
@@ -941,7 +941,7 @@
         <v>0.15999</v>
       </c>
       <c r="M10" s="16" t="n">
-        <v>1.77</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="11">
@@ -956,22 +956,22 @@
         </is>
       </c>
       <c r="C11" s="12" t="n">
-        <v>31.839873024</v>
+        <v>37.20300544</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>91.13</v>
+        <v>106.48</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>7.0099998</v>
+        <v>7.993994</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>9.21297</v>
+        <v>10.857916</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>1.316349967917976</v>
+        <v>1.538076957168844</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>1.316349967917976</v>
+        <v>1.538076957168844</v>
       </c>
       <c r="I11" s="15" t="n">
         <v>-0.033</v>
@@ -1001,37 +1001,37 @@
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>14.63074011428571</v>
+        <v>16.85456446171429</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>366.8785714285714</v>
+        <v>417.1128571428571</v>
       </c>
       <c r="E13" s="20" t="n">
-        <v>12.05149492857143</v>
+        <v>13.53908457142857</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>12.74192771428571</v>
+        <v>15.19152021428571</v>
       </c>
       <c r="G13" s="20" t="n">
-        <v>2.272205857434273</v>
+        <v>2.676560114466369</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>2.352573070768814</v>
+        <v>2.768250796923206</v>
       </c>
       <c r="I13" s="21" t="n">
-        <v>0.09385714285714285</v>
+        <v>0.1152857142857143</v>
       </c>
       <c r="J13" s="21" t="n">
-        <v>0.2021136293877293</v>
+        <v>0.2051600500990755</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>0.1964671594627567</v>
+        <v>0.1994809436539057</v>
       </c>
       <c r="L13" s="21" t="n">
-        <v>0.1896285714285715</v>
+        <v>0.1935228571428572</v>
       </c>
       <c r="M13" s="22" t="n">
-        <v>1.0025</v>
+        <v>0.8575</v>
       </c>
     </row>
     <row r="14">
@@ -1046,25 +1046,25 @@
         </is>
       </c>
       <c r="C14" s="18" t="n">
-        <v>7.338410496</v>
+        <v>8.792969215999999</v>
       </c>
       <c r="D14" s="19" t="n">
-        <v>99.54000000000001</v>
+        <v>119.27</v>
       </c>
       <c r="E14" s="20" t="n">
-        <v>13.244554</v>
+        <v>14.577198</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>13.998798</v>
+        <v>15.769044</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>2.581594676550765</v>
+        <v>2.901929292421108</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>2.63139683804179</v>
+        <v>2.957911105743479</v>
       </c>
       <c r="I14" s="21" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="J14" s="21" t="n">
         <v>0.2087421486045296</v>
@@ -1076,7 +1076,7 @@
         <v>0.20106001</v>
       </c>
       <c r="M14" s="22" t="n">
-        <v>0.96</v>
+        <v>0.8250000000000001</v>
       </c>
     </row>
     <row r="16">

</xml_diff>